<commit_message>
docs: added additional cases, automation pending
</commit_message>
<xml_diff>
--- a/test-cases.xlsx
+++ b/test-cases.xlsx
@@ -9,6 +9,7 @@
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="UI Tests" sheetId="1" state="visible" r:id="rId1"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="API Tests" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="AI Eval Tests" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -32,7 +33,7 @@
       <sz val="11"/>
     </font>
   </fonts>
-  <fills count="4">
+  <fills count="6">
     <fill>
       <patternFill/>
     </fill>
@@ -47,6 +48,16 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00EAF3FB"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="006B3FA0"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00F3EAFC"/>
       </patternFill>
     </fill>
   </fills>
@@ -76,7 +87,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
@@ -85,6 +96,12 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -452,7 +469,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H35"/>
+  <dimension ref="A1:H40"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -1935,6 +1952,216 @@
         </is>
       </c>
     </row>
+    <row r="36" ht="55" customHeight="1">
+      <c r="A36" s="2" t="inlineStr">
+        <is>
+          <t>UI035</t>
+        </is>
+      </c>
+      <c r="B36" s="2" t="inlineStr">
+        <is>
+          <t>menu.spec.js</t>
+        </is>
+      </c>
+      <c r="C36" s="2" t="inlineStr">
+        <is>
+          <t>GET /menu/abc returns 422 for non-integer ID</t>
+        </is>
+      </c>
+      <c r="D36" s="2" t="inlineStr">
+        <is>
+          <t>Navigate to frontend, menu loaded</t>
+        </is>
+      </c>
+      <c r="E36" s="2" t="inlineStr">
+        <is>
+          <t>Call GET /menu/abc directly via fetch</t>
+        </is>
+      </c>
+      <c r="F36" s="2" t="inlineStr">
+        <is>
+          <t>Response status is 422 Unprocessable Entity</t>
+        </is>
+      </c>
+      <c r="G36" s="2" t="inlineStr">
+        <is>
+          <t>422</t>
+        </is>
+      </c>
+      <c r="H36" s="2" t="inlineStr">
+        <is>
+          <t>Non-integer item ID should return 422 not 500</t>
+        </is>
+      </c>
+    </row>
+    <row r="37" ht="55" customHeight="1">
+      <c r="A37" s="3" t="inlineStr">
+        <is>
+          <t>UI036</t>
+        </is>
+      </c>
+      <c r="B37" s="3" t="inlineStr">
+        <is>
+          <t>order.spec.js</t>
+        </is>
+      </c>
+      <c r="C37" s="3" t="inlineStr">
+        <is>
+          <t>Negative quantity in order is rejected</t>
+        </is>
+      </c>
+      <c r="D37" s="3" t="inlineStr">
+        <is>
+          <t>Add item to cart, go to payment</t>
+        </is>
+      </c>
+      <c r="E37" s="3" t="inlineStr">
+        <is>
+          <t>Manually send POST /order with quantity -1 via fetch</t>
+        </is>
+      </c>
+      <c r="F37" s="3" t="inlineStr">
+        <is>
+          <t>Response status 400 or 422, error message shown</t>
+        </is>
+      </c>
+      <c r="G37" s="3" t="inlineStr">
+        <is>
+          <t>400 or 422</t>
+        </is>
+      </c>
+      <c r="H37" s="3" t="inlineStr">
+        <is>
+          <t>Negative quantity should be rejected with error</t>
+        </is>
+      </c>
+    </row>
+    <row r="38" ht="55" customHeight="1">
+      <c r="A38" s="2" t="inlineStr">
+        <is>
+          <t>UI037</t>
+        </is>
+      </c>
+      <c r="B38" s="2" t="inlineStr">
+        <is>
+          <t>order.spec.js</t>
+        </is>
+      </c>
+      <c r="C38" s="2" t="inlineStr">
+        <is>
+          <t>Zero quantity in order is rejected</t>
+        </is>
+      </c>
+      <c r="D38" s="2" t="inlineStr">
+        <is>
+          <t>Add item to cart</t>
+        </is>
+      </c>
+      <c r="E38" s="2" t="inlineStr">
+        <is>
+          <t>Manually send POST /order with quantity 0</t>
+        </is>
+      </c>
+      <c r="F38" s="2" t="inlineStr">
+        <is>
+          <t>Response status 400 or 422</t>
+        </is>
+      </c>
+      <c r="G38" s="2" t="inlineStr">
+        <is>
+          <t>400 or 422</t>
+        </is>
+      </c>
+      <c r="H38" s="2" t="inlineStr">
+        <is>
+          <t>Zero quantity should be rejected with error</t>
+        </is>
+      </c>
+    </row>
+    <row r="39" ht="55" customHeight="1">
+      <c r="A39" s="3" t="inlineStr">
+        <is>
+          <t>UI038</t>
+        </is>
+      </c>
+      <c r="B39" s="3" t="inlineStr">
+        <is>
+          <t>order.spec.js</t>
+        </is>
+      </c>
+      <c r="C39" s="3" t="inlineStr">
+        <is>
+          <t>Frontend shows error when order API fails</t>
+        </is>
+      </c>
+      <c r="D39" s="3" t="inlineStr">
+        <is>
+          <t>Add items to cart, mock /order to return 500</t>
+        </is>
+      </c>
+      <c r="E39" s="3" t="inlineStr">
+        <is>
+          <t>Click Place Order</t>
+        </is>
+      </c>
+      <c r="F39" s="3" t="inlineStr">
+        <is>
+          <t>Error message visible to user on screen</t>
+        </is>
+      </c>
+      <c r="G39" s="3" t="inlineStr">
+        <is>
+          <t>error message shown</t>
+        </is>
+      </c>
+      <c r="H39" s="3" t="inlineStr">
+        <is>
+          <t>Frontend must show user-friendly error when order API fails</t>
+        </is>
+      </c>
+    </row>
+    <row r="40" ht="55" customHeight="1">
+      <c r="A40" s="2" t="inlineStr">
+        <is>
+          <t>UI039</t>
+        </is>
+      </c>
+      <c r="B40" s="2" t="inlineStr">
+        <is>
+          <t>order.spec.js</t>
+        </is>
+      </c>
+      <c r="C40" s="2" t="inlineStr">
+        <is>
+          <t>Frontend shows error when payment API fails</t>
+        </is>
+      </c>
+      <c r="D40" s="2" t="inlineStr">
+        <is>
+          <t>Complete order flow, mock /payment to return 500</t>
+        </is>
+      </c>
+      <c r="E40" s="2" t="inlineStr">
+        <is>
+          <t>Click Pay Now</t>
+        </is>
+      </c>
+      <c r="F40" s="2" t="inlineStr">
+        <is>
+          <t>Error message visible to user on screen</t>
+        </is>
+      </c>
+      <c r="G40" s="2" t="inlineStr">
+        <is>
+          <t>error message shown</t>
+        </is>
+      </c>
+      <c r="H40" s="2" t="inlineStr">
+        <is>
+          <t>Frontend must show user-friendly error when payment API fails</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -1946,7 +2173,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I21"/>
+  <dimension ref="A1:I31"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -2947,6 +3174,1854 @@
         </is>
       </c>
     </row>
+    <row r="22" ht="55" customHeight="1">
+      <c r="A22" s="2" t="inlineStr">
+        <is>
+          <t>API021</t>
+        </is>
+      </c>
+      <c r="B22" s="2" t="inlineStr">
+        <is>
+          <t>api.spec.js</t>
+        </is>
+      </c>
+      <c r="C22" s="2" t="inlineStr">
+        <is>
+          <t>GET /menu/abc returns 422 for non-integer ID</t>
+        </is>
+      </c>
+      <c r="D22" s="2" t="inlineStr">
+        <is>
+          <t>GET</t>
+        </is>
+      </c>
+      <c r="E22" s="2" t="inlineStr">
+        <is>
+          <t>/menu/abc</t>
+        </is>
+      </c>
+      <c r="F22" s="2" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="G22" s="2" t="inlineStr">
+        <is>
+          <t>response.status()</t>
+        </is>
+      </c>
+      <c r="H22" s="2" t="inlineStr">
+        <is>
+          <t>422</t>
+        </is>
+      </c>
+      <c r="I22" s="2" t="inlineStr">
+        <is>
+          <t>Non-integer item ID should return 422 Unprocessable Entity</t>
+        </is>
+      </c>
+    </row>
+    <row r="23" ht="55" customHeight="1">
+      <c r="A23" s="3" t="inlineStr">
+        <is>
+          <t>API022</t>
+        </is>
+      </c>
+      <c r="B23" s="3" t="inlineStr">
+        <is>
+          <t>api.spec.js</t>
+        </is>
+      </c>
+      <c r="C23" s="3" t="inlineStr">
+        <is>
+          <t>POST order with negative quantity returns 400 or 422</t>
+        </is>
+      </c>
+      <c r="D23" s="3" t="inlineStr">
+        <is>
+          <t>POST</t>
+        </is>
+      </c>
+      <c r="E23" s="3" t="inlineStr">
+        <is>
+          <t>/order</t>
+        </is>
+      </c>
+      <c r="F23" s="3" t="inlineStr">
+        <is>
+          <t>{"items":[{"item_id":1,"quantity":-1}]}</t>
+        </is>
+      </c>
+      <c r="G23" s="3" t="inlineStr">
+        <is>
+          <t>response.status()</t>
+        </is>
+      </c>
+      <c r="H23" s="3" t="inlineStr">
+        <is>
+          <t>400 or 422</t>
+        </is>
+      </c>
+      <c r="I23" s="3" t="inlineStr">
+        <is>
+          <t>Negative quantity in order should be rejected</t>
+        </is>
+      </c>
+    </row>
+    <row r="24" ht="55" customHeight="1">
+      <c r="A24" s="2" t="inlineStr">
+        <is>
+          <t>API023</t>
+        </is>
+      </c>
+      <c r="B24" s="2" t="inlineStr">
+        <is>
+          <t>api.spec.js</t>
+        </is>
+      </c>
+      <c r="C24" s="2" t="inlineStr">
+        <is>
+          <t>POST order with zero quantity returns 400 or 422</t>
+        </is>
+      </c>
+      <c r="D24" s="2" t="inlineStr">
+        <is>
+          <t>POST</t>
+        </is>
+      </c>
+      <c r="E24" s="2" t="inlineStr">
+        <is>
+          <t>/order</t>
+        </is>
+      </c>
+      <c r="F24" s="2" t="inlineStr">
+        <is>
+          <t>{"items":[{"item_id":1,"quantity":0}]}</t>
+        </is>
+      </c>
+      <c r="G24" s="2" t="inlineStr">
+        <is>
+          <t>response.status()</t>
+        </is>
+      </c>
+      <c r="H24" s="2" t="inlineStr">
+        <is>
+          <t>400 or 422</t>
+        </is>
+      </c>
+      <c r="I24" s="2" t="inlineStr">
+        <is>
+          <t>Zero quantity in order should be rejected</t>
+        </is>
+      </c>
+    </row>
+    <row r="25" ht="55" customHeight="1">
+      <c r="A25" s="3" t="inlineStr">
+        <is>
+          <t>API024</t>
+        </is>
+      </c>
+      <c r="B25" s="3" t="inlineStr">
+        <is>
+          <t>api.spec.js</t>
+        </is>
+      </c>
+      <c r="C25" s="3" t="inlineStr">
+        <is>
+          <t>POST order with large quantity calculates total correctly</t>
+        </is>
+      </c>
+      <c r="D25" s="3" t="inlineStr">
+        <is>
+          <t>POST</t>
+        </is>
+      </c>
+      <c r="E25" s="3" t="inlineStr">
+        <is>
+          <t>/order</t>
+        </is>
+      </c>
+      <c r="F25" s="3" t="inlineStr">
+        <is>
+          <t>{"items":[{"item_id":1,"quantity":9999}]}</t>
+        </is>
+      </c>
+      <c r="G25" s="3" t="inlineStr">
+        <is>
+          <t>body.total</t>
+        </is>
+      </c>
+      <c r="H25" s="3" t="inlineStr">
+        <is>
+          <t>9999 x item price</t>
+        </is>
+      </c>
+      <c r="I25" s="3" t="inlineStr">
+        <is>
+          <t>Large quantity total should calculate correctly without overflow</t>
+        </is>
+      </c>
+    </row>
+    <row r="26" ht="55" customHeight="1">
+      <c r="A26" s="2" t="inlineStr">
+        <is>
+          <t>API025</t>
+        </is>
+      </c>
+      <c r="B26" s="2" t="inlineStr">
+        <is>
+          <t>api.spec.js</t>
+        </is>
+      </c>
+      <c r="C26" s="2" t="inlineStr">
+        <is>
+          <t>POST order with string item_id returns 422</t>
+        </is>
+      </c>
+      <c r="D26" s="2" t="inlineStr">
+        <is>
+          <t>POST</t>
+        </is>
+      </c>
+      <c r="E26" s="2" t="inlineStr">
+        <is>
+          <t>/order</t>
+        </is>
+      </c>
+      <c r="F26" s="2" t="inlineStr">
+        <is>
+          <t>{"items":[{"item_id":"abc","quantity":1}]}</t>
+        </is>
+      </c>
+      <c r="G26" s="2" t="inlineStr">
+        <is>
+          <t>response.status()</t>
+        </is>
+      </c>
+      <c r="H26" s="2" t="inlineStr">
+        <is>
+          <t>422</t>
+        </is>
+      </c>
+      <c r="I26" s="2" t="inlineStr">
+        <is>
+          <t>String item_id should return 422 Unprocessable Entity</t>
+        </is>
+      </c>
+    </row>
+    <row r="27" ht="55" customHeight="1">
+      <c r="A27" s="3" t="inlineStr">
+        <is>
+          <t>API026</t>
+        </is>
+      </c>
+      <c r="B27" s="3" t="inlineStr">
+        <is>
+          <t>api.spec.js</t>
+        </is>
+      </c>
+      <c r="C27" s="3" t="inlineStr">
+        <is>
+          <t>POST order with missing items field returns 422</t>
+        </is>
+      </c>
+      <c r="D27" s="3" t="inlineStr">
+        <is>
+          <t>POST</t>
+        </is>
+      </c>
+      <c r="E27" s="3" t="inlineStr">
+        <is>
+          <t>/order</t>
+        </is>
+      </c>
+      <c r="F27" s="3" t="inlineStr">
+        <is>
+          <t>{}</t>
+        </is>
+      </c>
+      <c r="G27" s="3" t="inlineStr">
+        <is>
+          <t>response.status()</t>
+        </is>
+      </c>
+      <c r="H27" s="3" t="inlineStr">
+        <is>
+          <t>422</t>
+        </is>
+      </c>
+      <c r="I27" s="3" t="inlineStr">
+        <is>
+          <t>Missing items field in order should return 422</t>
+        </is>
+      </c>
+    </row>
+    <row r="28" ht="55" customHeight="1">
+      <c r="A28" s="2" t="inlineStr">
+        <is>
+          <t>API027</t>
+        </is>
+      </c>
+      <c r="B28" s="2" t="inlineStr">
+        <is>
+          <t>api.spec.js</t>
+        </is>
+      </c>
+      <c r="C28" s="2" t="inlineStr">
+        <is>
+          <t>POST payment with negative amount returns failed status</t>
+        </is>
+      </c>
+      <c r="D28" s="2" t="inlineStr">
+        <is>
+          <t>POST</t>
+        </is>
+      </c>
+      <c r="E28" s="2" t="inlineStr">
+        <is>
+          <t>/payment</t>
+        </is>
+      </c>
+      <c r="F28" s="2" t="inlineStr">
+        <is>
+          <t>{"order_id":"test","amount":-100,"simulate_failure":false}</t>
+        </is>
+      </c>
+      <c r="G28" s="2" t="inlineStr">
+        <is>
+          <t>body.status</t>
+        </is>
+      </c>
+      <c r="H28" s="2" t="inlineStr">
+        <is>
+          <t>failed</t>
+        </is>
+      </c>
+      <c r="I28" s="2" t="inlineStr">
+        <is>
+          <t>Negative payment amount should return failed status</t>
+        </is>
+      </c>
+    </row>
+    <row r="29" ht="55" customHeight="1">
+      <c r="A29" s="3" t="inlineStr">
+        <is>
+          <t>API028</t>
+        </is>
+      </c>
+      <c r="B29" s="3" t="inlineStr">
+        <is>
+          <t>api.spec.js</t>
+        </is>
+      </c>
+      <c r="C29" s="3" t="inlineStr">
+        <is>
+          <t>POST payment with missing order_id returns 422</t>
+        </is>
+      </c>
+      <c r="D29" s="3" t="inlineStr">
+        <is>
+          <t>POST</t>
+        </is>
+      </c>
+      <c r="E29" s="3" t="inlineStr">
+        <is>
+          <t>/payment</t>
+        </is>
+      </c>
+      <c r="F29" s="3" t="inlineStr">
+        <is>
+          <t>{"amount":199,"simulate_failure":false}</t>
+        </is>
+      </c>
+      <c r="G29" s="3" t="inlineStr">
+        <is>
+          <t>response.status()</t>
+        </is>
+      </c>
+      <c r="H29" s="3" t="inlineStr">
+        <is>
+          <t>422</t>
+        </is>
+      </c>
+      <c r="I29" s="3" t="inlineStr">
+        <is>
+          <t>Missing order_id in payment should return 422</t>
+        </is>
+      </c>
+    </row>
+    <row r="30" ht="55" customHeight="1">
+      <c r="A30" s="2" t="inlineStr">
+        <is>
+          <t>API029</t>
+        </is>
+      </c>
+      <c r="B30" s="2" t="inlineStr">
+        <is>
+          <t>api.spec.js</t>
+        </is>
+      </c>
+      <c r="C30" s="2" t="inlineStr">
+        <is>
+          <t>POST payment with string amount returns 422</t>
+        </is>
+      </c>
+      <c r="D30" s="2" t="inlineStr">
+        <is>
+          <t>POST</t>
+        </is>
+      </c>
+      <c r="E30" s="2" t="inlineStr">
+        <is>
+          <t>/payment</t>
+        </is>
+      </c>
+      <c r="F30" s="2" t="inlineStr">
+        <is>
+          <t>{"order_id":"test","amount":"abc","simulate_failure":false}</t>
+        </is>
+      </c>
+      <c r="G30" s="2" t="inlineStr">
+        <is>
+          <t>response.status()</t>
+        </is>
+      </c>
+      <c r="H30" s="2" t="inlineStr">
+        <is>
+          <t>422</t>
+        </is>
+      </c>
+      <c r="I30" s="2" t="inlineStr">
+        <is>
+          <t>String amount in payment should return 422 Unprocessable Entity</t>
+        </is>
+      </c>
+    </row>
+    <row r="31" ht="55" customHeight="1">
+      <c r="A31" s="3" t="inlineStr">
+        <is>
+          <t>API030</t>
+        </is>
+      </c>
+      <c r="B31" s="3" t="inlineStr">
+        <is>
+          <t>api.spec.js</t>
+        </is>
+      </c>
+      <c r="C31" s="3" t="inlineStr">
+        <is>
+          <t>GET summary before any order placed returns 404</t>
+        </is>
+      </c>
+      <c r="D31" s="3" t="inlineStr">
+        <is>
+          <t>GET</t>
+        </is>
+      </c>
+      <c r="E31" s="3" t="inlineStr">
+        <is>
+          <t>/summary/nonexistent-order-id</t>
+        </is>
+      </c>
+      <c r="F31" s="3" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="G31" s="3" t="inlineStr">
+        <is>
+          <t>response.status()</t>
+        </is>
+      </c>
+      <c r="H31" s="3" t="inlineStr">
+        <is>
+          <t>404</t>
+        </is>
+      </c>
+      <c r="I31" s="3" t="inlineStr">
+        <is>
+          <t>Summary for non-existent order should return 404</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:J26"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="10" customWidth="1" min="1" max="1"/>
+    <col width="25" customWidth="1" min="2" max="2"/>
+    <col width="38" customWidth="1" min="3" max="3"/>
+    <col width="18" customWidth="1" min="4" max="4"/>
+    <col width="18" customWidth="1" min="5" max="5"/>
+    <col width="35" customWidth="1" min="6" max="6"/>
+    <col width="35" customWidth="1" min="7" max="7"/>
+    <col width="25" customWidth="1" min="8" max="8"/>
+    <col width="42" customWidth="1" min="9" max="9"/>
+    <col width="15" customWidth="1" min="10" max="10"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="30" customHeight="1">
+      <c r="A1" s="4" t="inlineStr">
+        <is>
+          <t>Test ID</t>
+        </is>
+      </c>
+      <c r="B1" s="4" t="inlineStr">
+        <is>
+          <t>Test File</t>
+        </is>
+      </c>
+      <c r="C1" s="4" t="inlineStr">
+        <is>
+          <t>Test Name</t>
+        </is>
+      </c>
+      <c r="D1" s="4" t="inlineStr">
+        <is>
+          <t>Component</t>
+        </is>
+      </c>
+      <c r="E1" s="4" t="inlineStr">
+        <is>
+          <t>Eval Tool</t>
+        </is>
+      </c>
+      <c r="F1" s="4" t="inlineStr">
+        <is>
+          <t>Input</t>
+        </is>
+      </c>
+      <c r="G1" s="4" t="inlineStr">
+        <is>
+          <t>What is Evaluated</t>
+        </is>
+      </c>
+      <c r="H1" s="4" t="inlineStr">
+        <is>
+          <t>Expected Result</t>
+        </is>
+      </c>
+      <c r="I1" s="4" t="inlineStr">
+        <is>
+          <t>Assert Message</t>
+        </is>
+      </c>
+      <c r="J1" s="4" t="inlineStr">
+        <is>
+          <t>Eval Layer</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="55" customHeight="1">
+      <c r="A2" s="5" t="inlineStr">
+        <is>
+          <t>AIE001</t>
+        </is>
+      </c>
+      <c r="B2" s="5" t="inlineStr">
+        <is>
+          <t>test_llm_eval.py</t>
+        </is>
+      </c>
+      <c r="C2" s="5" t="inlineStr">
+        <is>
+          <t>Summary contains correct order total</t>
+        </is>
+      </c>
+      <c r="D2" s="5" t="inlineStr">
+        <is>
+          <t>AI Summary</t>
+        </is>
+      </c>
+      <c r="E2" s="5" t="inlineStr">
+        <is>
+          <t>Custom pytest</t>
+        </is>
+      </c>
+      <c r="F2" s="5" t="inlineStr">
+        <is>
+          <t>Order with 1 Burger ₹199</t>
+        </is>
+      </c>
+      <c r="G2" s="5" t="inlineStr">
+        <is>
+          <t>Total amount ₹199 present in summary</t>
+        </is>
+      </c>
+      <c r="H2" s="5" t="inlineStr">
+        <is>
+          <t>₹199 in response</t>
+        </is>
+      </c>
+      <c r="I2" s="5" t="inlineStr">
+        <is>
+          <t>Summary must contain the correct total amount</t>
+        </is>
+      </c>
+      <c r="J2" s="5" t="inlineStr">
+        <is>
+          <t>Unit</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="55" customHeight="1">
+      <c r="A3" s="3" t="inlineStr">
+        <is>
+          <t>AIE002</t>
+        </is>
+      </c>
+      <c r="B3" s="3" t="inlineStr">
+        <is>
+          <t>test_llm_eval.py</t>
+        </is>
+      </c>
+      <c r="C3" s="3" t="inlineStr">
+        <is>
+          <t>Summary mentions all ordered item names</t>
+        </is>
+      </c>
+      <c r="D3" s="3" t="inlineStr">
+        <is>
+          <t>AI Summary</t>
+        </is>
+      </c>
+      <c r="E3" s="3" t="inlineStr">
+        <is>
+          <t>Custom pytest</t>
+        </is>
+      </c>
+      <c r="F3" s="3" t="inlineStr">
+        <is>
+          <t>Order with Burger</t>
+        </is>
+      </c>
+      <c r="G3" s="3" t="inlineStr">
+        <is>
+          <t>Item name present in summary</t>
+        </is>
+      </c>
+      <c r="H3" s="3" t="inlineStr">
+        <is>
+          <t>Item name present</t>
+        </is>
+      </c>
+      <c r="I3" s="3" t="inlineStr">
+        <is>
+          <t>Summary must mention every ordered item</t>
+        </is>
+      </c>
+      <c r="J3" s="3" t="inlineStr">
+        <is>
+          <t>Unit</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="55" customHeight="1">
+      <c r="A4" s="5" t="inlineStr">
+        <is>
+          <t>AIE003</t>
+        </is>
+      </c>
+      <c r="B4" s="5" t="inlineStr">
+        <is>
+          <t>test_llm_eval.py</t>
+        </is>
+      </c>
+      <c r="C4" s="5" t="inlineStr">
+        <is>
+          <t>Summary does not hallucinate unordered items</t>
+        </is>
+      </c>
+      <c r="D4" s="5" t="inlineStr">
+        <is>
+          <t>AI Summary</t>
+        </is>
+      </c>
+      <c r="E4" s="5" t="inlineStr">
+        <is>
+          <t>DeepEval Hallucination</t>
+        </is>
+      </c>
+      <c r="F4" s="5" t="inlineStr">
+        <is>
+          <t>Order with only Burger</t>
+        </is>
+      </c>
+      <c r="G4" s="5" t="inlineStr">
+        <is>
+          <t>No unordered items mentioned</t>
+        </is>
+      </c>
+      <c r="H4" s="5" t="inlineStr">
+        <is>
+          <t>No hallucinated items</t>
+        </is>
+      </c>
+      <c r="I4" s="5" t="inlineStr">
+        <is>
+          <t>Summary must not mention items not in the order</t>
+        </is>
+      </c>
+      <c r="J4" s="5" t="inlineStr">
+        <is>
+          <t>Unit</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="55" customHeight="1">
+      <c r="A5" s="3" t="inlineStr">
+        <is>
+          <t>AIE004</t>
+        </is>
+      </c>
+      <c r="B5" s="3" t="inlineStr">
+        <is>
+          <t>test_llm_eval.py</t>
+        </is>
+      </c>
+      <c r="C5" s="3" t="inlineStr">
+        <is>
+          <t>Summary does not invent prices</t>
+        </is>
+      </c>
+      <c r="D5" s="3" t="inlineStr">
+        <is>
+          <t>AI Summary</t>
+        </is>
+      </c>
+      <c r="E5" s="3" t="inlineStr">
+        <is>
+          <t>Custom pytest</t>
+        </is>
+      </c>
+      <c r="F5" s="3" t="inlineStr">
+        <is>
+          <t>Order with Burger ₹199</t>
+        </is>
+      </c>
+      <c r="G5" s="3" t="inlineStr">
+        <is>
+          <t>No price other than ₹199 appears</t>
+        </is>
+      </c>
+      <c r="H5" s="3" t="inlineStr">
+        <is>
+          <t>Correct price only</t>
+        </is>
+      </c>
+      <c r="I5" s="3" t="inlineStr">
+        <is>
+          <t>Summary must not contain invented price values</t>
+        </is>
+      </c>
+      <c r="J5" s="3" t="inlineStr">
+        <is>
+          <t>Unit</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="55" customHeight="1">
+      <c r="A6" s="5" t="inlineStr">
+        <is>
+          <t>AIE005</t>
+        </is>
+      </c>
+      <c r="B6" s="5" t="inlineStr">
+        <is>
+          <t>test_llm_eval.py</t>
+        </is>
+      </c>
+      <c r="C6" s="5" t="inlineStr">
+        <is>
+          <t>Every fact grounded in order data</t>
+        </is>
+      </c>
+      <c r="D6" s="5" t="inlineStr">
+        <is>
+          <t>AI Summary</t>
+        </is>
+      </c>
+      <c r="E6" s="5" t="inlineStr">
+        <is>
+          <t>DeepEval Faithfulness</t>
+        </is>
+      </c>
+      <c r="F6" s="5" t="inlineStr">
+        <is>
+          <t>Order dict</t>
+        </is>
+      </c>
+      <c r="G6" s="5" t="inlineStr">
+        <is>
+          <t>All claims traceable to order</t>
+        </is>
+      </c>
+      <c r="H6" s="5" t="inlineStr">
+        <is>
+          <t>Faithfulness &gt;= 0.8</t>
+        </is>
+      </c>
+      <c r="I6" s="5" t="inlineStr">
+        <is>
+          <t>Summary must be faithful to order data</t>
+        </is>
+      </c>
+      <c r="J6" s="5" t="inlineStr">
+        <is>
+          <t>Unit</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="55" customHeight="1">
+      <c r="A7" s="3" t="inlineStr">
+        <is>
+          <t>AIE006</t>
+        </is>
+      </c>
+      <c r="B7" s="3" t="inlineStr">
+        <is>
+          <t>test_llm_eval.py</t>
+        </is>
+      </c>
+      <c r="C7" s="3" t="inlineStr">
+        <is>
+          <t>Summary does not invent delivery time</t>
+        </is>
+      </c>
+      <c r="D7" s="3" t="inlineStr">
+        <is>
+          <t>AI Summary</t>
+        </is>
+      </c>
+      <c r="E7" s="3" t="inlineStr">
+        <is>
+          <t>Custom pytest</t>
+        </is>
+      </c>
+      <c r="F7" s="3" t="inlineStr">
+        <is>
+          <t>Standard order</t>
+        </is>
+      </c>
+      <c r="G7" s="3" t="inlineStr">
+        <is>
+          <t>No delivery time mentioned</t>
+        </is>
+      </c>
+      <c r="H7" s="3" t="inlineStr">
+        <is>
+          <t>No invented ETA</t>
+        </is>
+      </c>
+      <c r="I7" s="3" t="inlineStr">
+        <is>
+          <t>Summary must not mention invented delivery time</t>
+        </is>
+      </c>
+      <c r="J7" s="3" t="inlineStr">
+        <is>
+          <t>Unit</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="55" customHeight="1">
+      <c r="A8" s="5" t="inlineStr">
+        <is>
+          <t>AIE007</t>
+        </is>
+      </c>
+      <c r="B8" s="5" t="inlineStr">
+        <is>
+          <t>test_llm_eval.py</t>
+        </is>
+      </c>
+      <c r="C8" s="5" t="inlineStr">
+        <is>
+          <t>Summary relevant to food order confirmation</t>
+        </is>
+      </c>
+      <c r="D8" s="5" t="inlineStr">
+        <is>
+          <t>AI Summary</t>
+        </is>
+      </c>
+      <c r="E8" s="5" t="inlineStr">
+        <is>
+          <t>DeepEval Relevancy</t>
+        </is>
+      </c>
+      <c r="F8" s="5" t="inlineStr">
+        <is>
+          <t>Order context</t>
+        </is>
+      </c>
+      <c r="G8" s="5" t="inlineStr">
+        <is>
+          <t>Response about food order</t>
+        </is>
+      </c>
+      <c r="H8" s="5" t="inlineStr">
+        <is>
+          <t>Relevancy &gt;= 0.8</t>
+        </is>
+      </c>
+      <c r="I8" s="5" t="inlineStr">
+        <is>
+          <t>Summary must be relevant to food order</t>
+        </is>
+      </c>
+      <c r="J8" s="5" t="inlineStr">
+        <is>
+          <t>Unit</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="55" customHeight="1">
+      <c r="A9" s="3" t="inlineStr">
+        <is>
+          <t>AIE008</t>
+        </is>
+      </c>
+      <c r="B9" s="3" t="inlineStr">
+        <is>
+          <t>test_llm_eval.py</t>
+        </is>
+      </c>
+      <c r="C9" s="3" t="inlineStr">
+        <is>
+          <t>Summary stays on topic</t>
+        </is>
+      </c>
+      <c r="D9" s="3" t="inlineStr">
+        <is>
+          <t>AI Summary</t>
+        </is>
+      </c>
+      <c r="E9" s="3" t="inlineStr">
+        <is>
+          <t>Custom pytest</t>
+        </is>
+      </c>
+      <c r="F9" s="3" t="inlineStr">
+        <is>
+          <t>Standard order</t>
+        </is>
+      </c>
+      <c r="G9" s="3" t="inlineStr">
+        <is>
+          <t>No unrelated content</t>
+        </is>
+      </c>
+      <c r="H9" s="3" t="inlineStr">
+        <is>
+          <t>On topic</t>
+        </is>
+      </c>
+      <c r="I9" s="3" t="inlineStr">
+        <is>
+          <t>Summary must not contain unrelated content</t>
+        </is>
+      </c>
+      <c r="J9" s="3" t="inlineStr">
+        <is>
+          <t>Unit</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="55" customHeight="1">
+      <c r="A10" s="5" t="inlineStr">
+        <is>
+          <t>AIE009</t>
+        </is>
+      </c>
+      <c r="B10" s="5" t="inlineStr">
+        <is>
+          <t>test_llm_eval.py</t>
+        </is>
+      </c>
+      <c r="C10" s="5" t="inlineStr">
+        <is>
+          <t>Summary includes closing message</t>
+        </is>
+      </c>
+      <c r="D10" s="5" t="inlineStr">
+        <is>
+          <t>AI Summary</t>
+        </is>
+      </c>
+      <c r="E10" s="5" t="inlineStr">
+        <is>
+          <t>Custom pytest</t>
+        </is>
+      </c>
+      <c r="F10" s="5" t="inlineStr">
+        <is>
+          <t>Standard order</t>
+        </is>
+      </c>
+      <c r="G10" s="5" t="inlineStr">
+        <is>
+          <t>Closing statement present</t>
+        </is>
+      </c>
+      <c r="H10" s="5" t="inlineStr">
+        <is>
+          <t>Closing present</t>
+        </is>
+      </c>
+      <c r="I10" s="5" t="inlineStr">
+        <is>
+          <t>Summary must include friendly closing</t>
+        </is>
+      </c>
+      <c r="J10" s="5" t="inlineStr">
+        <is>
+          <t>Unit</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="55" customHeight="1">
+      <c r="A11" s="3" t="inlineStr">
+        <is>
+          <t>AIE010</t>
+        </is>
+      </c>
+      <c r="B11" s="3" t="inlineStr">
+        <is>
+          <t>test_llm_eval.py</t>
+        </is>
+      </c>
+      <c r="C11" s="3" t="inlineStr">
+        <is>
+          <t>Summary is 2 to 4 sentences</t>
+        </is>
+      </c>
+      <c r="D11" s="3" t="inlineStr">
+        <is>
+          <t>AI Summary</t>
+        </is>
+      </c>
+      <c r="E11" s="3" t="inlineStr">
+        <is>
+          <t>Custom pytest</t>
+        </is>
+      </c>
+      <c r="F11" s="3" t="inlineStr">
+        <is>
+          <t>Standard order</t>
+        </is>
+      </c>
+      <c r="G11" s="3" t="inlineStr">
+        <is>
+          <t>Sentence count 2-4</t>
+        </is>
+      </c>
+      <c r="H11" s="3" t="inlineStr">
+        <is>
+          <t>2-4 sentences</t>
+        </is>
+      </c>
+      <c r="I11" s="3" t="inlineStr">
+        <is>
+          <t>Summary length must match instructions</t>
+        </is>
+      </c>
+      <c r="J11" s="3" t="inlineStr">
+        <is>
+          <t>Unit</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="55" customHeight="1">
+      <c r="A12" s="5" t="inlineStr">
+        <is>
+          <t>AIE011</t>
+        </is>
+      </c>
+      <c r="B12" s="5" t="inlineStr">
+        <is>
+          <t>test_llm_eval.py</t>
+        </is>
+      </c>
+      <c r="C12" s="5" t="inlineStr">
+        <is>
+          <t>Summary is plain text no JSON or code</t>
+        </is>
+      </c>
+      <c r="D12" s="5" t="inlineStr">
+        <is>
+          <t>AI Summary</t>
+        </is>
+      </c>
+      <c r="E12" s="5" t="inlineStr">
+        <is>
+          <t>Custom pytest</t>
+        </is>
+      </c>
+      <c r="F12" s="5" t="inlineStr">
+        <is>
+          <t>Standard order</t>
+        </is>
+      </c>
+      <c r="G12" s="5" t="inlineStr">
+        <is>
+          <t>No braces or code syntax</t>
+        </is>
+      </c>
+      <c r="H12" s="5" t="inlineStr">
+        <is>
+          <t>Plain text only</t>
+        </is>
+      </c>
+      <c r="I12" s="5" t="inlineStr">
+        <is>
+          <t>Summary must be plain readable text</t>
+        </is>
+      </c>
+      <c r="J12" s="5" t="inlineStr">
+        <is>
+          <t>Unit</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="55" customHeight="1">
+      <c r="A13" s="3" t="inlineStr">
+        <is>
+          <t>AIE012</t>
+        </is>
+      </c>
+      <c r="B13" s="3" t="inlineStr">
+        <is>
+          <t>test_llm_eval.py</t>
+        </is>
+      </c>
+      <c r="C13" s="3" t="inlineStr">
+        <is>
+          <t>Summary contains no markdown</t>
+        </is>
+      </c>
+      <c r="D13" s="3" t="inlineStr">
+        <is>
+          <t>AI Summary</t>
+        </is>
+      </c>
+      <c r="E13" s="3" t="inlineStr">
+        <is>
+          <t>Custom pytest</t>
+        </is>
+      </c>
+      <c r="F13" s="3" t="inlineStr">
+        <is>
+          <t>Standard order</t>
+        </is>
+      </c>
+      <c r="G13" s="3" t="inlineStr">
+        <is>
+          <t>No markdown symbols</t>
+        </is>
+      </c>
+      <c r="H13" s="3" t="inlineStr">
+        <is>
+          <t>No markdown</t>
+        </is>
+      </c>
+      <c r="I13" s="3" t="inlineStr">
+        <is>
+          <t>Summary must not contain markdown</t>
+        </is>
+      </c>
+      <c r="J13" s="3" t="inlineStr">
+        <is>
+          <t>Unit</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="55" customHeight="1">
+      <c r="A14" s="5" t="inlineStr">
+        <is>
+          <t>AIE013</t>
+        </is>
+      </c>
+      <c r="B14" s="5" t="inlineStr">
+        <is>
+          <t>test_llm_eval.py</t>
+        </is>
+      </c>
+      <c r="C14" s="5" t="inlineStr">
+        <is>
+          <t>Summary is in English</t>
+        </is>
+      </c>
+      <c r="D14" s="5" t="inlineStr">
+        <is>
+          <t>AI Summary</t>
+        </is>
+      </c>
+      <c r="E14" s="5" t="inlineStr">
+        <is>
+          <t>Custom pytest</t>
+        </is>
+      </c>
+      <c r="F14" s="5" t="inlineStr">
+        <is>
+          <t>Standard order</t>
+        </is>
+      </c>
+      <c r="G14" s="5" t="inlineStr">
+        <is>
+          <t>English language detected</t>
+        </is>
+      </c>
+      <c r="H14" s="5" t="inlineStr">
+        <is>
+          <t>English</t>
+        </is>
+      </c>
+      <c r="I14" s="5" t="inlineStr">
+        <is>
+          <t>Summary must be in English</t>
+        </is>
+      </c>
+      <c r="J14" s="5" t="inlineStr">
+        <is>
+          <t>Unit</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="55" customHeight="1">
+      <c r="A15" s="3" t="inlineStr">
+        <is>
+          <t>AIE014</t>
+        </is>
+      </c>
+      <c r="B15" s="3" t="inlineStr">
+        <is>
+          <t>test_llm_eval.py</t>
+        </is>
+      </c>
+      <c r="C15" s="3" t="inlineStr">
+        <is>
+          <t>Summary contains no toxic content</t>
+        </is>
+      </c>
+      <c r="D15" s="3" t="inlineStr">
+        <is>
+          <t>AI Summary</t>
+        </is>
+      </c>
+      <c r="E15" s="3" t="inlineStr">
+        <is>
+          <t>DeepEval Toxicity</t>
+        </is>
+      </c>
+      <c r="F15" s="3" t="inlineStr">
+        <is>
+          <t>Standard order</t>
+        </is>
+      </c>
+      <c r="G15" s="3" t="inlineStr">
+        <is>
+          <t>No harmful language</t>
+        </is>
+      </c>
+      <c r="H15" s="3" t="inlineStr">
+        <is>
+          <t>Toxicity &lt; 0.1</t>
+        </is>
+      </c>
+      <c r="I15" s="3" t="inlineStr">
+        <is>
+          <t>Summary must be free of toxic content</t>
+        </is>
+      </c>
+      <c r="J15" s="3" t="inlineStr">
+        <is>
+          <t>Unit</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="55" customHeight="1">
+      <c r="A16" s="5" t="inlineStr">
+        <is>
+          <t>AIE015</t>
+        </is>
+      </c>
+      <c r="B16" s="5" t="inlineStr">
+        <is>
+          <t>test_llm_eval.py</t>
+        </is>
+      </c>
+      <c r="C16" s="5" t="inlineStr">
+        <is>
+          <t>Summary contains no PII</t>
+        </is>
+      </c>
+      <c r="D16" s="5" t="inlineStr">
+        <is>
+          <t>AI Summary</t>
+        </is>
+      </c>
+      <c r="E16" s="5" t="inlineStr">
+        <is>
+          <t>Custom pytest</t>
+        </is>
+      </c>
+      <c r="F16" s="5" t="inlineStr">
+        <is>
+          <t>Order without PII</t>
+        </is>
+      </c>
+      <c r="G16" s="5" t="inlineStr">
+        <is>
+          <t>No email or phone in response</t>
+        </is>
+      </c>
+      <c r="H16" s="5" t="inlineStr">
+        <is>
+          <t>No PII</t>
+        </is>
+      </c>
+      <c r="I16" s="5" t="inlineStr">
+        <is>
+          <t>Summary must not expose personal information</t>
+        </is>
+      </c>
+      <c r="J16" s="5" t="inlineStr">
+        <is>
+          <t>Unit</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="55" customHeight="1">
+      <c r="A17" s="3" t="inlineStr">
+        <is>
+          <t>AIE016</t>
+        </is>
+      </c>
+      <c r="B17" s="3" t="inlineStr">
+        <is>
+          <t>test_llm_eval.py</t>
+        </is>
+      </c>
+      <c r="C17" s="3" t="inlineStr">
+        <is>
+          <t>AI summary returns within 15 seconds</t>
+        </is>
+      </c>
+      <c r="D17" s="3" t="inlineStr">
+        <is>
+          <t>AI Summary</t>
+        </is>
+      </c>
+      <c r="E17" s="3" t="inlineStr">
+        <is>
+          <t>Custom pytest time.time()</t>
+        </is>
+      </c>
+      <c r="F17" s="3" t="inlineStr">
+        <is>
+          <t>Standard order</t>
+        </is>
+      </c>
+      <c r="G17" s="3" t="inlineStr">
+        <is>
+          <t>Response time &lt; 15s</t>
+        </is>
+      </c>
+      <c r="H17" s="3" t="inlineStr">
+        <is>
+          <t>&lt; 15 seconds</t>
+        </is>
+      </c>
+      <c r="I17" s="3" t="inlineStr">
+        <is>
+          <t>AI summary must return within acceptable latency</t>
+        </is>
+      </c>
+      <c r="J17" s="3" t="inlineStr">
+        <is>
+          <t>Unit</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="55" customHeight="1">
+      <c r="A18" s="5" t="inlineStr">
+        <is>
+          <t>AIE017</t>
+        </is>
+      </c>
+      <c r="B18" s="5" t="inlineStr">
+        <is>
+          <t>ai_eval.spec.js</t>
+        </is>
+      </c>
+      <c r="C18" s="5" t="inlineStr">
+        <is>
+          <t>AI summary appears in UI within 15 seconds</t>
+        </is>
+      </c>
+      <c r="D18" s="5" t="inlineStr">
+        <is>
+          <t>AI Summary UI</t>
+        </is>
+      </c>
+      <c r="E18" s="5" t="inlineStr">
+        <is>
+          <t>Playwright waitForSelector</t>
+        </is>
+      </c>
+      <c r="F18" s="5" t="inlineStr">
+        <is>
+          <t>Full order flow</t>
+        </is>
+      </c>
+      <c r="G18" s="5" t="inlineStr">
+        <is>
+          <t>Summary visible within 15s</t>
+        </is>
+      </c>
+      <c r="H18" s="5" t="inlineStr">
+        <is>
+          <t>visible within 15s</t>
+        </is>
+      </c>
+      <c r="I18" s="5" t="inlineStr">
+        <is>
+          <t>AI summary must appear in UI within acceptable time</t>
+        </is>
+      </c>
+      <c r="J18" s="5" t="inlineStr">
+        <is>
+          <t>E2E</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="55" customHeight="1">
+      <c r="A19" s="3" t="inlineStr">
+        <is>
+          <t>AIE018</t>
+        </is>
+      </c>
+      <c r="B19" s="3" t="inlineStr">
+        <is>
+          <t>test_llm_eval.py</t>
+        </is>
+      </c>
+      <c r="C19" s="3" t="inlineStr">
+        <is>
+          <t>Fallback triggers when API key missing</t>
+        </is>
+      </c>
+      <c r="D19" s="3" t="inlineStr">
+        <is>
+          <t>AI Summary</t>
+        </is>
+      </c>
+      <c r="E19" s="3" t="inlineStr">
+        <is>
+          <t>Custom pytest</t>
+        </is>
+      </c>
+      <c r="F19" s="3" t="inlineStr">
+        <is>
+          <t>Invalid API key</t>
+        </is>
+      </c>
+      <c r="G19" s="3" t="inlineStr">
+        <is>
+          <t>Fallback message returned</t>
+        </is>
+      </c>
+      <c r="H19" s="3" t="inlineStr">
+        <is>
+          <t>Fallback returned</t>
+        </is>
+      </c>
+      <c r="I19" s="3" t="inlineStr">
+        <is>
+          <t>System must return fallback gracefully</t>
+        </is>
+      </c>
+      <c r="J19" s="3" t="inlineStr">
+        <is>
+          <t>Unit</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="55" customHeight="1">
+      <c r="A20" s="5" t="inlineStr">
+        <is>
+          <t>AIE019</t>
+        </is>
+      </c>
+      <c r="B20" s="5" t="inlineStr">
+        <is>
+          <t>test_llm_eval.py</t>
+        </is>
+      </c>
+      <c r="C20" s="5" t="inlineStr">
+        <is>
+          <t>Fallback contains correct total</t>
+        </is>
+      </c>
+      <c r="D20" s="5" t="inlineStr">
+        <is>
+          <t>AI Summary</t>
+        </is>
+      </c>
+      <c r="E20" s="5" t="inlineStr">
+        <is>
+          <t>Custom pytest</t>
+        </is>
+      </c>
+      <c r="F20" s="5" t="inlineStr">
+        <is>
+          <t>Invalid API key, order ₹199</t>
+        </is>
+      </c>
+      <c r="G20" s="5" t="inlineStr">
+        <is>
+          <t>Fallback contains ₹199</t>
+        </is>
+      </c>
+      <c r="H20" s="5" t="inlineStr">
+        <is>
+          <t>Correct total in fallback</t>
+        </is>
+      </c>
+      <c r="I20" s="5" t="inlineStr">
+        <is>
+          <t>Fallback must show correct order total</t>
+        </is>
+      </c>
+      <c r="J20" s="5" t="inlineStr">
+        <is>
+          <t>Unit</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="55" customHeight="1">
+      <c r="A21" s="3" t="inlineStr">
+        <is>
+          <t>AIE020</t>
+        </is>
+      </c>
+      <c r="B21" s="3" t="inlineStr">
+        <is>
+          <t>test_llm_eval.py</t>
+        </is>
+      </c>
+      <c r="C21" s="3" t="inlineStr">
+        <is>
+          <t>Fallback is user friendly</t>
+        </is>
+      </c>
+      <c r="D21" s="3" t="inlineStr">
+        <is>
+          <t>AI Summary</t>
+        </is>
+      </c>
+      <c r="E21" s="3" t="inlineStr">
+        <is>
+          <t>Custom pytest</t>
+        </is>
+      </c>
+      <c r="F21" s="3" t="inlineStr">
+        <is>
+          <t>Invalid API key</t>
+        </is>
+      </c>
+      <c r="G21" s="3" t="inlineStr">
+        <is>
+          <t>No error details exposed</t>
+        </is>
+      </c>
+      <c r="H21" s="3" t="inlineStr">
+        <is>
+          <t>User friendly text</t>
+        </is>
+      </c>
+      <c r="I21" s="3" t="inlineStr">
+        <is>
+          <t>Fallback must not expose internal errors</t>
+        </is>
+      </c>
+      <c r="J21" s="3" t="inlineStr">
+        <is>
+          <t>Unit</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" ht="55" customHeight="1">
+      <c r="A22" s="5" t="inlineStr">
+        <is>
+          <t>AIE021</t>
+        </is>
+      </c>
+      <c r="B22" s="5" t="inlineStr">
+        <is>
+          <t>test_llm_eval.py</t>
+        </is>
+      </c>
+      <c r="C22" s="5" t="inlineStr">
+        <is>
+          <t>Same order produces relevant summary 3 runs</t>
+        </is>
+      </c>
+      <c r="D22" s="5" t="inlineStr">
+        <is>
+          <t>AI Summary</t>
+        </is>
+      </c>
+      <c r="E22" s="5" t="inlineStr">
+        <is>
+          <t>Custom pytest 3 runs</t>
+        </is>
+      </c>
+      <c r="F22" s="5" t="inlineStr">
+        <is>
+          <t>Same order 3 times</t>
+        </is>
+      </c>
+      <c r="G22" s="5" t="inlineStr">
+        <is>
+          <t>All 3 relevant and correct</t>
+        </is>
+      </c>
+      <c r="H22" s="5" t="inlineStr">
+        <is>
+          <t>3/3 pass</t>
+        </is>
+      </c>
+      <c r="I22" s="5" t="inlineStr">
+        <is>
+          <t>AI must consistently produce relevant output</t>
+        </is>
+      </c>
+      <c r="J22" s="5" t="inlineStr">
+        <is>
+          <t>Unit</t>
+        </is>
+      </c>
+    </row>
+    <row r="23" ht="55" customHeight="1">
+      <c r="A23" s="3" t="inlineStr">
+        <is>
+          <t>AIE022</t>
+        </is>
+      </c>
+      <c r="B23" s="3" t="inlineStr">
+        <is>
+          <t>test_llm_eval.py</t>
+        </is>
+      </c>
+      <c r="C23" s="3" t="inlineStr">
+        <is>
+          <t>Total always present across 3 runs</t>
+        </is>
+      </c>
+      <c r="D23" s="3" t="inlineStr">
+        <is>
+          <t>AI Summary</t>
+        </is>
+      </c>
+      <c r="E23" s="3" t="inlineStr">
+        <is>
+          <t>Custom pytest 3 runs</t>
+        </is>
+      </c>
+      <c r="F23" s="3" t="inlineStr">
+        <is>
+          <t>Same order 3 times</t>
+        </is>
+      </c>
+      <c r="G23" s="3" t="inlineStr">
+        <is>
+          <t>All 3 contain total</t>
+        </is>
+      </c>
+      <c r="H23" s="3" t="inlineStr">
+        <is>
+          <t>3/3 contain total</t>
+        </is>
+      </c>
+      <c r="I23" s="3" t="inlineStr">
+        <is>
+          <t>Total must appear consistently</t>
+        </is>
+      </c>
+      <c r="J23" s="3" t="inlineStr">
+        <is>
+          <t>Unit</t>
+        </is>
+      </c>
+    </row>
+    <row r="24" ht="55" customHeight="1">
+      <c r="A24" s="5" t="inlineStr">
+        <is>
+          <t>AIE023</t>
+        </is>
+      </c>
+      <c r="B24" s="5" t="inlineStr">
+        <is>
+          <t>test_llm_eval.py</t>
+        </is>
+      </c>
+      <c r="C24" s="5" t="inlineStr">
+        <is>
+          <t>Coverage analyzer returns at least one gap</t>
+        </is>
+      </c>
+      <c r="D24" s="5" t="inlineStr">
+        <is>
+          <t>Coverage Analyzer</t>
+        </is>
+      </c>
+      <c r="E24" s="5" t="inlineStr">
+        <is>
+          <t>Custom pytest</t>
+        </is>
+      </c>
+      <c r="F24" s="5" t="inlineStr">
+        <is>
+          <t>Sample pytest output</t>
+        </is>
+      </c>
+      <c r="G24" s="5" t="inlineStr">
+        <is>
+          <t>At least one gap identified</t>
+        </is>
+      </c>
+      <c r="H24" s="5" t="inlineStr">
+        <is>
+          <t>1+ gaps</t>
+        </is>
+      </c>
+      <c r="I24" s="5" t="inlineStr">
+        <is>
+          <t>Analyzer must identify missing scenarios</t>
+        </is>
+      </c>
+      <c r="J24" s="5" t="inlineStr">
+        <is>
+          <t>Unit</t>
+        </is>
+      </c>
+    </row>
+    <row r="25" ht="55" customHeight="1">
+      <c r="A25" s="3" t="inlineStr">
+        <is>
+          <t>AIE024</t>
+        </is>
+      </c>
+      <c r="B25" s="3" t="inlineStr">
+        <is>
+          <t>test_llm_eval.py</t>
+        </is>
+      </c>
+      <c r="C25" s="3" t="inlineStr">
+        <is>
+          <t>Coverage analyzer is actionable LLM as Judge</t>
+        </is>
+      </c>
+      <c r="D25" s="3" t="inlineStr">
+        <is>
+          <t>Coverage Analyzer</t>
+        </is>
+      </c>
+      <c r="E25" s="3" t="inlineStr">
+        <is>
+          <t>LLM-as-a-Judge GPT-4o-mini</t>
+        </is>
+      </c>
+      <c r="F25" s="3" t="inlineStr">
+        <is>
+          <t>Sample pytest output</t>
+        </is>
+      </c>
+      <c r="G25" s="3" t="inlineStr">
+        <is>
+          <t>Judge scores &gt;= 7/10</t>
+        </is>
+      </c>
+      <c r="H25" s="3" t="inlineStr">
+        <is>
+          <t>Score &gt;= 7</t>
+        </is>
+      </c>
+      <c r="I25" s="3" t="inlineStr">
+        <is>
+          <t>Analyzer output must be specific and actionable</t>
+        </is>
+      </c>
+      <c r="J25" s="3" t="inlineStr">
+        <is>
+          <t>Unit</t>
+        </is>
+      </c>
+    </row>
+    <row r="26" ht="55" customHeight="1">
+      <c r="A26" s="5" t="inlineStr">
+        <is>
+          <t>AIE025</t>
+        </is>
+      </c>
+      <c r="B26" s="5" t="inlineStr">
+        <is>
+          <t>test_llm_eval.py</t>
+        </is>
+      </c>
+      <c r="C26" s="5" t="inlineStr">
+        <is>
+          <t>Coverage analyzer fallback when API unavailable</t>
+        </is>
+      </c>
+      <c r="D26" s="5" t="inlineStr">
+        <is>
+          <t>Coverage Analyzer</t>
+        </is>
+      </c>
+      <c r="E26" s="5" t="inlineStr">
+        <is>
+          <t>Custom pytest</t>
+        </is>
+      </c>
+      <c r="F26" s="5" t="inlineStr">
+        <is>
+          <t>Invalid API key</t>
+        </is>
+      </c>
+      <c r="G26" s="5" t="inlineStr">
+        <is>
+          <t>Fallback returned gracefully</t>
+        </is>
+      </c>
+      <c r="H26" s="5" t="inlineStr">
+        <is>
+          <t>Fallback returned</t>
+        </is>
+      </c>
+      <c r="I26" s="5" t="inlineStr">
+        <is>
+          <t>Analyzer must degrade gracefully</t>
+        </is>
+      </c>
+      <c r="J26" s="5" t="inlineStr">
+        <is>
+          <t>Unit</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>